<commit_message>
3rd changes to set framwork aftet BD referech Nov 3 2023
</commit_message>
<xml_diff>
--- a/TestData/TMTI0045469_VerifyNewTitleAddedinTitleRateSheet.xlsx
+++ b/TestData/TMTI0045469_VerifyNewTitleAddedinTitleRateSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VKumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D5AB9D-41BB-4B3F-BB6D-18E8602E2580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{918F142A-DE3D-423B-ADC2-EA35EAD9B6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Global Search User</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>DRC - Original</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
 </sst>
 </file>
@@ -407,7 +410,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FC3538F-EBF7-4442-B955-CB25CC734266}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -416,7 +419,7 @@
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -430,7 +433,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -441,6 +444,9 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>